<commit_message>
fix: DDR5 차트 CSV 같은 날 세션 갱신 + 일일 데이터 갱신 + mezzanine_cache.json git 추적 제거 (100MB 초과, 로컬 전용)
- DDR5: 11시 세션 값 고정으로 캡션과 차트 끝점 불일치 해소, 과거 6개 행 치유
- 백필로 캐시가 157MB로 커져 GitHub 한도 초과 → .gitignore 추가

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data_us/us_disclosures_summary_20260707.xlsx
+++ b/data_us/us_disclosures_summary_20260707.xlsx
@@ -19,7 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'자금조달'!$A$1:$H$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'계약_사업'!$A$1:$H$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'M&amp;A_경영권'!$A$1:$H$32</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'5%지분'!$A$1:$H$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'5%지분'!$A$1:$K$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'경영진변동'!$A$1:$H$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'실적_정기'!$A$1:$H$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'리스크신호'!$A$1:$H$2</definedName>
@@ -95,7 +95,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -107,8 +107,17 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -480,12 +489,12 @@
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="44" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="70" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -521,7 +530,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>설명</t>
+          <t>핵심내용</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -559,8 +568,12 @@
           <t>발행조건 확정</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr"/>
-      <c r="H2" s="5" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>Amazon.com, Inc.는 변동금리부 채권(Compounded SOFR + 스프레드, 분기 이자 지급)과 7종의 고정금리부 채권(각각 이자율·만기일 공란)을 발행하는 예비신고서를 제출했으며, 각 트랜치별 발행액과 이자율은 아직 확정되지 않았다(금액 미정).</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -595,8 +608,12 @@
           <t>발행조건 확정</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>AutoZone, Inc.는 원금액, 이자율, 만기일이 모두 공란인 선순위 무담보 사채를 발행하는 예비신고서를 제출했으며, 구체적 조건은 추후 확정될 예정이다(금액 미정).</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -631,8 +648,12 @@
           <t>[2.03] 채무 발생(차입·사채)</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>MasTec과 MasTec North America는 Bank of America를 주관사로 하여 총 7억 달러(3년물 4억 달러, 4년물 3억 달러)의 선인출 조건부 기한부 대출 약정을 체결했으며, 인수대금 및 관련 비용 조달이 목적이다.</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -667,12 +688,12 @@
           <t>발행조건 확정</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>DEAL 1154</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Jefferies Financial Group Inc.는 2026년 7월 8일 만기(가치평가일 2032년 7월 2일)의 원금 2,932,000달러, 액면 1,000달러당 조건부 쿠폰 16.08달러를 지급하는 선순위 무담보 자동콜 조건부 쿠폰 배리어 어음(기초자산: Nasdaq-100, Russell 2000, VanEck 반도체 ETF 중 최저 성과)을 발행한다.</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -701,12 +722,12 @@
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="44" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="70" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -742,7 +763,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>설명</t>
+          <t>핵심내용</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -780,8 +801,12 @@
           <t>[1.01] 주요 계약 체결</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr"/>
-      <c r="H2" s="5" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>Vertex Pharmaceuticals가 2026년 7월 6일 Crinetics Pharmaceuticals를 인수하는 합병계약을 체결했으며, 합병 후 Crinetics는 Vertex의 완전 자회사로 존속한다. (금액 미정)</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -816,8 +841,12 @@
           <t>[1.01] 주요 계약 체결</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>MasTec과 MasTec North America는 Bank of America를 주관사로 하여 총 7억 달러(3년물 4억 달러, 4년물 3억 달러)의 선인출 조건부 기한부 대출 약정을 체결했으며, 인수대금 및 관련 비용 조달이 목적이다.</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -844,12 +873,12 @@
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="44" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="70" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -885,7 +914,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>설명</t>
+          <t>핵심내용</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -923,8 +952,12 @@
           <t>합병 관련 커뮤니케이션</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr"/>
-      <c r="H2" s="5" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>GameStop Corp.의 CEO Ryan Cohen은 2026년 5월 eBay의 모든 발행 보통주를 주당 125달러(현금 50%, GameStop 보통주 50%)에 인수하는 제안을 했으나, eBay 이사회는 2026년 5월 12일 이를 거절했다.</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -959,8 +992,12 @@
           <t>합병 관련 커뮤니케이션</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>GameStop Corp. 이사 Larry Cheng은 GameStop이 약 560억 달러 규모의 eBay 인수 제안을 했으며, eBay 이사회가 이를 거절했지만 GameStop은 여전히 거래를 추진할 의향이 있다고 밝혔다.</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -995,8 +1032,12 @@
           <t>합병 관련 커뮤니케이션</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Fox Corporation의 Roku 인수와 관련하여, Roku 주주는 거래 종결 시 주당 96.00달러 현금과 Fox Class A 보통주 0.9693주를 받게 되며, 미행사 RSU는 동일한 조건의 현금 기반 보상과 Fox RSU로 전환된다.</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -1031,8 +1072,12 @@
           <t>합병 관련 커뮤니케이션</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Solstice Advanced Materials Inc.는 2026년 7월 6일, Element Solutions Inc.와 합병 계약을 체결했으며, 자회사인 Merger Sub One이 Element Solutions와 합병한 후, 그 존속법인이 다시 Merger Sub Two와 합병하여 Solstice의 완전 자회사가 되는 2단계 합병 구조이다.</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -1067,8 +1112,12 @@
           <t>공개매수(제3자)(정정)</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>GSK plc의 자회사 Harmony Row Acquisition Co.가 Nuvalent, Inc.의 보통주(Class A 및 Class B)를 주당 124.00달러에 전량 현금 매수하는 공개매수 정정신고서다.</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -1103,8 +1152,12 @@
           <t>공개매수 의견표명(정정)</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Nuvalent, Inc.은 Harmony Row Acquisition Co.(GSK plc의 간접 자회사)의 공개매수에 대해 주당 124.00달러(현금)에 모든 발행 보통주를 매수하는 조건에 대한 의견표명 정정 공시를 제출했으며, 공시 이후 11건의 주주 요청서를 수령했다.</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -1139,8 +1192,12 @@
           <t>합병 관련 커뮤니케이션</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr"/>
-      <c r="H8" s="5" t="inlineStr">
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Solstice Advanced Materials Inc.가 2026년 7월 7일 직원 타운홀에서 Element Solutions Inc와의 제안된 거래에 관한 프레젠테이션을 제공했다. (금액 미정)</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -1175,8 +1232,12 @@
           <t>합병 관련 커뮤니케이션</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr"/>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>Solstice Advanced Materials Inc가 2026년 7월 6일 Element Solutions Inc 인수 합의를 발표했으며, 관련 합병 관련 공동 투자자 콜의 녹취록이 제출되었다. (금액 미정)</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -1211,8 +1272,12 @@
           <t>합병 관련 커뮤니케이션</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr"/>
-      <c r="H10" s="5" t="inlineStr">
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>Solstice Advanced Materials Inc.가 Element Solutions Inc를 인수하는 계약을 체결했으며, 거래는 2027년 상반기 중 주주 및 규제 승인 등을 조건으로 종료될 예정이다.</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -1247,8 +1312,12 @@
           <t>합병 관련 커뮤니케이션</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr"/>
-      <c r="H11" s="5" t="inlineStr">
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>Solstice가 Element Solutions 인수를 위한 최종 계약을 체결했으며, 거래는 2027년 상반기 중 주주 및 규제 승인 등을 조건으로 종료될 예정이다.</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -1283,8 +1352,12 @@
           <t>합병 관련 커뮤니케이션</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr"/>
-      <c r="H12" s="5" t="inlineStr">
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>Solstice가 Element Solutions 인수를 위한 최종 계약을 체결했으며, 거래는 2027년 상반기 중 양사 주주 및 규제 승인 등을 조건으로 종료될 예정이다.</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -1319,8 +1392,8 @@
           <t>합병 관련 커뮤니케이션</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr"/>
-      <c r="H13" s="5" t="inlineStr">
+      <c r="G13" s="5" t="inlineStr"/>
+      <c r="H13" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -1355,8 +1428,8 @@
           <t>합병 관련 커뮤니케이션</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr"/>
-      <c r="H14" s="5" t="inlineStr">
+      <c r="G14" s="5" t="inlineStr"/>
+      <c r="H14" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -1391,8 +1464,12 @@
           <t>합병 관련 커뮤니케이션</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr"/>
-      <c r="H15" s="5" t="inlineStr">
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>Element Solutions Inc가 Solstice Advanced Materials와의 결합을 발표했으며, Element의 CEO Ben Gliklich는 일상 경영에서 물러나 Solstice 이사회 멤버로 활동할 예정이다.</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -1427,8 +1504,12 @@
           <t>합병 관련 커뮤니케이션</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr"/>
-      <c r="H16" s="5" t="inlineStr">
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>Iridium Communications Inc.가 자회사를 통해 Aireon Holdings LLC의 기존 미보유 지분 61%를 약 3억 6670만 달러에 인수 완료했으며, 대금의 50%는 현금, 나머지는 무이자 1년 만기 대출(1억 8336만 달러)로 지급했다.</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -1440,31 +1521,29 @@
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>OLPX</t>
-        </is>
-      </c>
+      <c r="B17" s="2" t="inlineStr"/>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>OLAPLEX HOLDINGS, INC.; Nasdaq Stock Market LLC</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="n">
-        <v>1.4</v>
-      </c>
+          <t>Barings Private Credit Corp</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="n"/>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>25-NSE</t>
+          <t>SC TO-I/A</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>상장폐지(거래소)</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="inlineStr"/>
-      <c r="H17" s="5" t="inlineStr">
+          <t>공개매수(자사)(정정)</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>Barings Private Credit Corporation이 자사 보통주 최대 7,320,222주를 2026년 6월 30일 기준 순자산가치로 매수하는 자사주 공개매수 정정신고서다.</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -1479,22 +1558,26 @@
       <c r="B18" s="2" t="inlineStr"/>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Barings Private Credit Corp</t>
+          <t>BBR ALO Fund, LLC</t>
         </is>
       </c>
       <c r="D18" s="4" t="n"/>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>SC TO-I/A</t>
+          <t>SC TO-I</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>공개매수(자사)(정정)</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr"/>
-      <c r="H18" s="5" t="inlineStr">
+          <t>공개매수(자사)</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>BBR ALO Fund, LLC가 자사 지분증권을 최대 75,000,000달러 한도로 매수하는 자사 공개매수(2026년 9월 16일 만료)를 개시했다.</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -1509,7 +1592,7 @@
       <c r="B19" s="2" t="inlineStr"/>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>BBR ALO Fund, LLC</t>
+          <t>Constitution Capital Access Fund, LLC</t>
         </is>
       </c>
       <c r="D19" s="4" t="n"/>
@@ -1523,8 +1606,12 @@
           <t>공개매수(자사)</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr"/>
-      <c r="H19" s="5" t="inlineStr">
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>Constitution Capital Access Fund, LLC가 자사 순자산의 약 5.00%(약 39,484,825달러 또는 3,218,235주, 2026년 5월 31일 기준)를 순자산가치로 매수하는 자사 공개매수를 개시했다.</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -1539,22 +1626,22 @@
       <c r="B20" s="2" t="inlineStr"/>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Constitution Capital Access Fund, LLC</t>
+          <t>Rome Wildlife, Inc.</t>
         </is>
       </c>
       <c r="D20" s="4" t="n"/>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>SC TO-I</t>
+          <t>S-4/A</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>공개매수(자사)</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr"/>
-      <c r="H20" s="5" t="inlineStr">
+          <t>합병·교환 증권등록(정정)</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr"/>
+      <c r="H20" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -1569,22 +1656,26 @@
       <c r="B21" s="2" t="inlineStr"/>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Rome Wildlife, Inc.</t>
+          <t>Alternative Credit Income Fund</t>
         </is>
       </c>
       <c r="D21" s="4" t="n"/>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>S-4/A</t>
+          <t>425</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>합병·교환 증권등록(정정)</t>
-        </is>
-      </c>
-      <c r="G21" s="3" t="inlineStr"/>
-      <c r="H21" s="5" t="inlineStr">
+          <t>합병 관련 커뮤니케이션</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>Alternative Credit Income Fund(ACIF)는 BC Partners Lending Corporation(BCPL) 자회사와의 합병안 승인을 위한 임시 주주총회를 2026년 7월 7일에서 8월 14일로 연기했으며, 2026년 7월 6일 기준 주주 투표의 약 87%가 합병에 찬성했다.</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -1613,8 +1704,12 @@
           <t>합병 관련 커뮤니케이션</t>
         </is>
       </c>
-      <c r="G22" s="3" t="inlineStr"/>
-      <c r="H22" s="5" t="inlineStr">
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>Alternative Credit Income Fund(ACIF)는 BC Partners Lending Corporation(BCPL) 자회사와의 합병안 승인을 위한 임시 주주총회를 2026년 7월 7일에서 8월 14일로 연기했으며, 2026년 7월 6일 기준 주주 투표의 약 87%가 합병에 찬성했다.</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -1643,8 +1738,12 @@
           <t>합병 관련 커뮤니케이션</t>
         </is>
       </c>
-      <c r="G23" s="3" t="inlineStr"/>
-      <c r="H23" s="5" t="inlineStr">
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>Alternative Credit Income Fund가 합병 관련 커뮤니케이션을 SEC에 제출했으며, 관련 등록명세서 파일 번호는 333-294601이다. (금액 미정)</t>
+        </is>
+      </c>
+      <c r="H23" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -1659,7 +1758,7 @@
       <c r="B24" s="2" t="inlineStr"/>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Alternative Credit Income Fund</t>
+          <t>Pasqal Holding SAS; Bleichroeder Acquisition France Merger Sub 2</t>
         </is>
       </c>
       <c r="D24" s="4" t="n"/>
@@ -1673,8 +1772,12 @@
           <t>합병 관련 커뮤니케이션</t>
         </is>
       </c>
-      <c r="G24" s="3" t="inlineStr"/>
-      <c r="H24" s="5" t="inlineStr">
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>Pasqal과 MegazoneCloud가 한국에서 산업용 양자 컴퓨팅 도입을 위해 양해각서(MoU)를 체결했으며, Pasqal의 QPU를 MegazoneCloud 관리형 클라우드 서비스에 통합하고 국내 고객 대상 온프레미스 QPU 배포 기회를 추진한다. (금액 미정)</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -1689,7 +1792,7 @@
       <c r="B25" s="2" t="inlineStr"/>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Pasqal Holding SAS; Bleichroeder Acquisition France Merger Sub 2</t>
+          <t>Evernorth Holdings Inc.</t>
         </is>
       </c>
       <c r="D25" s="4" t="n"/>
@@ -1703,8 +1806,12 @@
           <t>합병 관련 커뮤니케이션</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr"/>
-      <c r="H25" s="5" t="inlineStr">
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>Evernorth Holdings Inc.가 SPAC인 Armada Acquisition Corp. II와의 사업 결합 관련 등록명세서(예비 위임장/투자설명서 포함)를 2026년 3월 18일 SEC에 제출했으나 아직 효력이 발생하지 않았다.</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -1719,22 +1826,22 @@
       <c r="B26" s="2" t="inlineStr"/>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Evernorth Holdings Inc.</t>
+          <t>Assertio Holdings, Inc.; Nasdaq Stock Market LLC</t>
         </is>
       </c>
       <c r="D26" s="4" t="n"/>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>425</t>
+          <t>25-NSE</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>합병 관련 커뮤니케이션</t>
-        </is>
-      </c>
-      <c r="G26" s="3" t="inlineStr"/>
-      <c r="H26" s="5" t="inlineStr">
+          <t>상장폐지(거래소)</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr"/>
+      <c r="H26" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -1749,7 +1856,7 @@
       <c r="B27" s="2" t="inlineStr"/>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Assertio Holdings, Inc.; Nasdaq Stock Market LLC</t>
+          <t>OLAPLEX HOLDINGS, INC.; Nasdaq Stock Market LLC</t>
         </is>
       </c>
       <c r="D27" s="4" t="n"/>
@@ -1763,8 +1870,8 @@
           <t>상장폐지(거래소)</t>
         </is>
       </c>
-      <c r="G27" s="3" t="inlineStr"/>
-      <c r="H27" s="5" t="inlineStr">
+      <c r="G27" s="5" t="inlineStr"/>
+      <c r="H27" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -1793,8 +1900,8 @@
           <t>상장폐지(거래소)</t>
         </is>
       </c>
-      <c r="G28" s="3" t="inlineStr"/>
-      <c r="H28" s="5" t="inlineStr">
+      <c r="G28" s="5" t="inlineStr"/>
+      <c r="H28" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -1827,8 +1934,12 @@
           <t>합병 주총 위임장</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr"/>
-      <c r="H29" s="5" t="inlineStr">
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>D. Boral ARC Acquisition I Corp.는 Exascale Labs Inc.와의 합병을 위한 주주총회 위임장을 제출했으며, 합병 후 존속법인(Exascale Labs Holdings Inc.)의 Class A 보통주 최대 60,456,000주, Class B 슈퍼 보통주 30,744,000주, 그리고 Class A 보통주 매수권 14,100,000주를 발행할 예정이다.</t>
+        </is>
+      </c>
+      <c r="H29" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -1863,8 +1974,12 @@
           <t>합병 관련 커뮤니케이션</t>
         </is>
       </c>
-      <c r="G30" s="3" t="inlineStr"/>
-      <c r="H30" s="5" t="inlineStr">
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>Onconetix, Inc.가 인수 예정인 Realbotix LLC가 Bloom Procurement Services와 협력하여 영국 북동부 요양 시설 노인 대상 사회적 돌봄 인간형 로봇 파일럿 프로그램을 시작했으며, Realbotix는 Bloom의 공공 부문 마켓플레이스 공급업체로 인증받았다. (금액 미정)</t>
+        </is>
+      </c>
+      <c r="H30" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -1897,8 +2012,12 @@
           <t>합병 관련 커뮤니케이션</t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr"/>
-      <c r="H31" s="5" t="inlineStr">
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t>Spring Valley Acquisition Corp. III는 2026년 7월 6일 주주 투표를 통해 General Fusion Inc.와의 사업 결합을 승인했으며, 거래 완료 후 합병 법인은 나스닥에서 "GFUZ"로 거래될 예정이다.</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -1931,8 +2050,12 @@
           <t>합병 관련 커뮤니케이션</t>
         </is>
       </c>
-      <c r="G32" s="3" t="inlineStr"/>
-      <c r="H32" s="5" t="inlineStr">
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>Spring Valley Acquisition Corp. III 주주들이 General Fusion Inc.와의 사업 결합을 승인했으며, 거래 종결은 2026년 7월 10일경 예정이고, 합병 후 법인은 나스닥에서 티커 "GFUZ"로 거래될 예정이다.</t>
+        </is>
+      </c>
+      <c r="H32" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -1983,17 +2106,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="44" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="70" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2029,10 +2155,25 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>설명</t>
+          <t>신고자</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>보유비율(%)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>보유주식수</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>핵심내용</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>링크</t>
         </is>
@@ -2067,8 +2208,23 @@
           <t>5% 보유 변동(경영참여)</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr"/>
-      <c r="H2" s="5" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>FRANKLIN RESOURCES INC, JOHNSON CHARLES B 외</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="n">
+        <v>68.7</v>
+      </c>
+      <c r="I2" s="8" t="n">
+        <v>75000</v>
+      </c>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>Holdco와 FRI는 발행인의 투자 전략 지원을 위해 주식을 취득했으며, 현재 증권 추가 취득·처분 계획이나 Item 4 (a)~(j)에 해당하는 계획은 없음.</t>
+        </is>
+      </c>
+      <c r="K2" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -2103,8 +2259,23 @@
           <t>5% 보유 변동(경영참여)</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>XP Control LLC, Guilherme Dias Fernandes Benchimol</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="I3" s="8" t="n">
+        <v>96797602</v>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>2026년 7월 2일 XP Control LLC가 매입권을 행사하여 Gabriel이 간접 보유한 비의결권 지분 전부를 4,954,867주의 클래스 A 보통주로 매입했고, 이에 따라 보고자의 클래스 A 보통주 보유 수는 101,752,469주에서 96,797,602주로 감소했으며, 추가로 최대 2,815,465주까지 감소할 수 있다.</t>
+        </is>
+      </c>
+      <c r="K3" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -2139,8 +2310,23 @@
           <t>5% 보유 변동(경영참여)</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Prescott General Partners LLC, Prescott Associates L.P. 외</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="I4" s="8" t="n">
+        <v>1427060</v>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>PGP가 파트너십을 통해 1,427,060주, PIPS가 직원 이익공유제 참가자 계좌로 41,437주, Smith와 Vassalluzzo가 각각 관리계좌를 통해 83,123주와 2,758주를 실질 보유하며, 총 관리계좌 보유 주식은 1,554,378주임.</t>
+        </is>
+      </c>
+      <c r="K4" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -2175,8 +2361,23 @@
           <t>5% 보유 변동(경영참여)</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Kamal Seyed Ghaffarian, Ghaffarian Enterprises, LLC 외</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="n">
+        <v>19.7</v>
+      </c>
+      <c r="I5" s="8" t="n">
+        <v>38429036</v>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>Intuitive Machines의 Ghaffarian Enterprises, LLC는 2026년 7월 2일 Rule 10b5-1에 따른 거래계획을 체결하여, 중개인을 통해 Class A 보통주 최대 1,935,568주(발행주식 총수의 2% 미만)를 유동성 확보 목적으로 매도할 예정이다.</t>
+        </is>
+      </c>
+      <c r="K5" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -2211,8 +2412,19 @@
           <t>5% 보유 변동(경영참여)</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Allseas Group S.A., Allseas Investments S.A. 외</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="I6" s="8" t="n">
+        <v>67502501</v>
+      </c>
+      <c r="J6" s="5" t="inlineStr"/>
+      <c r="K6" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -2247,8 +2459,23 @@
           <t>5% 보유 변동(경영참여)</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Sands Capital Life Sciences Pulse Fund II, L.P., Sands Capital Alternatives, LLC 외</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="I7" s="8" t="n">
+        <v>4230926</v>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>Alamar Biosciences의 보고자는 투자 목적으로 보통주를 보유하며, Ian Ratcliffe가 2026년 7월 5일 사망하여 이사회에서 물러났고 현재 다른 임원은 이사회에 참여하지 않으며 대표권을 추구할 계획이 없다.</t>
+        </is>
+      </c>
+      <c r="K7" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -2283,8 +2510,23 @@
           <t>5% 보유 변동(경영참여)</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr"/>
-      <c r="H8" s="5" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Prescott General Partners LLC, Prescott Associates L.P. 외</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="I8" s="8" t="n">
+        <v>1456150</v>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>PGP가 파트너십을 통해 1,456,150주, PIPS가 직원 이익공유제 참가자 계좌로 50,286주, Smith와 Vassalluzzo가 각각 관리계좌를 통해 71,150주와 1,788주를 실질 보유하며, 총 관리계좌 보유 주식은 1,579,374주임.</t>
+        </is>
+      </c>
+      <c r="K8" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -2319,8 +2561,23 @@
           <t>5% 보유 변동(경영참여)</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr"/>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>RA Capital Management, L.P., Peter Kolchinsky 외</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="n">
+        <v>33</v>
+      </c>
+      <c r="I9" s="8" t="n">
+        <v>23249186</v>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>Climb Bio의 보고자인 RA Capital은 2026년 6월 29일부로 애널리스트 Breanna Celebi(O'Reilly)를 이사로 지명하여 Andrew Levin을 교체했다.</t>
+        </is>
+      </c>
+      <c r="K9" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -2355,8 +2612,19 @@
           <t>5% 보유 변동(경영참여)</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr"/>
-      <c r="H10" s="5" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Legion Partners, L.P. I, Legion Partners, L.P. II 외</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="I10" s="8" t="n">
+        <v>4997847</v>
+      </c>
+      <c r="J10" s="5" t="inlineStr"/>
+      <c r="K10" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -2391,8 +2659,19 @@
           <t>5% 보유 변동(경영참여)</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr"/>
-      <c r="H11" s="5" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Oasis Management Co Ltd., Oasis Investments II Master Fund Ltd. 외</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="I11" s="8" t="n">
+        <v>843517</v>
+      </c>
+      <c r="J11" s="5" t="inlineStr"/>
+      <c r="K11" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -2427,8 +2706,23 @@
           <t>5% 보유 변동(경영참여)</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr"/>
-      <c r="H12" s="5" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Energy Evolution Master Fund, Ltd.</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="n">
+        <v>30.7</v>
+      </c>
+      <c r="I12" s="8" t="n">
+        <v>12209953</v>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>Energy Evolution Fund(EEF)는 보통주, 전환사채, 워런트를 투자 목적으로 취득·보유 중이며, 현재 Item 4 (a)~(j)에 해당하는 구체적 계획은 없으나 상황에 따라 보유 규모를 변경할 수 있음.</t>
+        </is>
+      </c>
+      <c r="K12" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -2463,8 +2757,23 @@
           <t>5% 이상 취득(경영참여)</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr"/>
-      <c r="H13" s="5" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Russell C. Horowitz</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="I13" s="8" t="n">
+        <v>8813485</v>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>보고자는 향후 Marchex 주식을 추가 매수하거나 전부 또는 일부를 처분할 수 있으나, 현재로서는 Schedule 13D Item 4의 (a)~(j)에 해당하는 구체적인 계획이나 제안은 없다.</t>
+        </is>
+      </c>
+      <c r="K13" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -2499,8 +2808,23 @@
           <t>5% 보유 변동(경영참여)</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr"/>
-      <c r="H14" s="5" t="inlineStr">
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>SCLX Stock Acquisition JV LLC</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="I14" s="8" t="n">
+        <v>30029378</v>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>2025년 4월 15일 발행사가 1:35 비율의 주식병합을 실시했고, 2026년 7월 3일 보고자는 발행사 보통주 500,000주를 Quantum Scan Holdings, Inc.에 이전하고 Q Scan의 보통주와 교환했으며, 이전 가격은 이전 직전 거래일의 나스닥 종가를 기준으로 한다.</t>
+        </is>
+      </c>
+      <c r="K14" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -2529,8 +2853,23 @@
           <t>5% 보유 변동(경영참여)</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr"/>
-      <c r="H15" s="5" t="inlineStr">
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Daniel Oliver Jr, Myrmikan Gold Fund, LLC 외</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="n">
+        <v>13.95</v>
+      </c>
+      <c r="I15" s="8" t="n">
+        <v>18108768</v>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>보고자 Oliver Daniel Jr.는 발행인 Rise Gold Corp.의 보통주 가치 극대화를 목표로 정책에 영향력을 행사하려 하며, 필요시 정기 주주총회 이사 후보 지명 과정에 참여할 수 있다.</t>
+        </is>
+      </c>
+      <c r="K15" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -2559,8 +2898,23 @@
           <t>5% 보유 변동(경영참여)</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr"/>
-      <c r="H16" s="5" t="inlineStr">
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>UAW Retiree Medical Benefits Trust, UAW Chrysler Retirees Medical Benefits Plan 외</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="n">
+        <v>99</v>
+      </c>
+      <c r="I16" s="8" t="n">
+        <v>620852</v>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>2025년 9월 29일(주당 915.86달러), 2025년 12월 29일(주당 909.79달러), 2026년 3월 30일(주당 895.75달러), 2026년 6월 26일(주당 882.50달러)에 각각 배당금 재투자 계획에 따라 UAW Chrysler, Ford, GM 퇴직자 의료급여 플랜에 각각 342.584주·534.080주·880.178주, 464.438주·724.047주·1,193.249주, 362.716주·565.465주·931.901주, 369.271주·575.685주·948.743주가 발행되었다.</t>
+        </is>
+      </c>
+      <c r="K16" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -2589,8 +2943,23 @@
           <t>5% 이상 취득(경영참여)</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr"/>
-      <c r="H17" s="5" t="inlineStr">
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>John P Calamos, Sr., Calamos Advisors LLC 외</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="n">
+        <v>16.2</v>
+      </c>
+      <c r="I17" s="8" t="n">
+        <v>950844</v>
+      </c>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>보고자는 Class I 주식을 투자 목적으로 취득·보유 중이며, 현재 Item 4 (a)~(j)에 해당하는 계획이나 제안은 없음.</t>
+        </is>
+      </c>
+      <c r="K17" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -2625,8 +2994,23 @@
           <t>5% 보유 변동(경영참여)</t>
         </is>
       </c>
-      <c r="G18" s="3" t="inlineStr"/>
-      <c r="H18" s="5" t="inlineStr">
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>Agriculture Investment Group Corp., Granosur Holding Limited</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="n">
+        <v>5.83</v>
+      </c>
+      <c r="I18" s="8" t="n">
+        <v>3722732</v>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>Bioceres Crop Solutions의 보고자는 현재 Item 4 (a)~(j)에 해당하는 구체적 계획이나 제안이 없으며, 향후 언제든지 입장을 재검토·변경할 수 있다.</t>
+        </is>
+      </c>
+      <c r="K18" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -2661,8 +3045,23 @@
           <t>5% 보유 변동(경영참여)</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr"/>
-      <c r="H19" s="5" t="inlineStr">
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Camac Partners, LLC, Camac Capital, LLC 외</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="I19" s="8" t="n">
+        <v>551081</v>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>CRYO CELL INTERNATIONAL의 보고자는 발행인의 증권이 저평가되었다고 판단하여 매수했으며, 향후 공개시장 또는 사적 거래를 통해 포지션을 늘리거나 줄일 수 있고, 이사회 구성·지출 수준·자산 현금화·주주 자본환원 등에 대해 경영진 및 이사회와 논의할 의사가 있다.</t>
+        </is>
+      </c>
+      <c r="K19" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -2695,8 +3094,23 @@
           <t>5% 이상 취득(경영참여)</t>
         </is>
       </c>
-      <c r="G20" s="3" t="inlineStr"/>
-      <c r="H20" s="5" t="inlineStr">
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>Osprey Acquisition Sponsor III, LLC, Hepco Capital Management, LLC 외</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="n">
+        <v>26.18</v>
+      </c>
+      <c r="I20" s="8" t="n">
+        <v>10740000</v>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>스폰서는 2026년 2월 2일 제공 비용 25,000달러를 지불했고, 2026년 5월에 25,000주를 반납하여 총 10,254,000주의 설립자주를 보유하게 되었으며, IPO 완료와 동시에 486,000개의 플레이스먼트 유닛을 유닛당 10.00달러에 매입했고, 각 유닛은 클래스 A 주식 1주와 11.50달러에 행사 가능한 워런트 1/3개로 구성된다.</t>
+        </is>
+      </c>
+      <c r="K20" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -2731,36 +3145,47 @@
           <t>5% 보유 변동(경영참여)</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr"/>
-      <c r="H21" s="5" t="inlineStr">
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>Hyperscale Data, Inc., Alpha Structured Finance LP 외</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="I21" s="8" t="n">
+        <v>319917</v>
+      </c>
+      <c r="J21" s="5" t="inlineStr"/>
+      <c r="K21" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H21"/>
+  <autoFilter ref="A1:K21"/>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K21" r:id="rId20"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2777,12 +3202,12 @@
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="44" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="70" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2818,7 +3243,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>설명</t>
+          <t>핵심내용</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -2856,8 +3281,8 @@
           <t>[5.02] 임원·이사 선임/사임</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr"/>
-      <c r="H2" s="5" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr"/>
+      <c r="H2" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -2892,8 +3317,8 @@
           <t>[5.02] 임원·이사 선임/사임</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -2928,8 +3353,12 @@
           <t>[5.02] 임원·이사 선임/사임</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>EchoStar Corporation 및 Hughes Satellite Systems Corporation의 CEO Hamid Akhavan이 2026년 7월 6일 이사회와의 전략 방향 논의 후 즉시 모든 직책에서 사임했음.</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -2964,8 +3393,12 @@
           <t>[5.02] 임원·이사 선임/사임</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>MasTec, Inc.와 자회사 MasTec North America가 2026년 7월 7일 Bank of America 등을 상대로 총 7억 달러(3년물 4억 달러, 4년물 3억 달러)의 신규 선순위 무담보 유예인출 기한부 대출 계약을 체결했으며, 인수대금 및 관련 비용 조달에 사용될 예정.</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -3000,8 +3433,12 @@
           <t>[5.02] 임원·이사 선임/사임</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Fiserv, Inc.의 사장 Dhivya Suryadevara가 2026년 7월 7일 고용계약상 '정당한 사유'로 사임했음.</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -3031,12 +3468,12 @@
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="44" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="70" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3072,7 +3509,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>설명</t>
+          <t>핵심내용</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -3110,8 +3547,12 @@
           <t>[2.02] 실적 발표</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr"/>
-      <c r="H2" s="5" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>ResMed Inc.가 2026년 6월 30일 MatrixCare 사업을 Frazier Healthcare Partners에 4억 9천만 달러 전액 현금 거래로 매각하는 최종 계약을 체결했으며, 해당 사업은 FY2026 기준 약 2억 2천만 달러 매출과 약 5천 5백만 달러 비GAAP 영업이익을 기록함.</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -3146,8 +3587,12 @@
           <t>[2.02] 실적 발표</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>DigitalOcean Holdings, Inc.가 2026년 7월 7일, 2026년 6월 30일 종료 분기의 잠정 미감사 재무 결과를 발표했다고 공시함 (구체적 수치 미기재).</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>
@@ -3174,12 +3619,12 @@
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="44" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="70" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3215,7 +3660,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>설명</t>
+          <t>핵심내용</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -3253,8 +3698,8 @@
           <t>[2.05] 구조조정 비용</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr"/>
-      <c r="H2" s="5" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr"/>
+      <c r="H2" s="6" t="inlineStr">
         <is>
           <t>EDGAR</t>
         </is>

</xml_diff>